<commit_message>
Using app reference metrics for final display values in case some blanks appear
</commit_message>
<xml_diff>
--- a/data/results/calculated_green_metrics.xlsx
+++ b/data/results/calculated_green_metrics.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N11"/>
+  <dimension ref="A1:X12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -439,52 +439,102 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>atom_economy_percent</t>
+          <t>display_atom_economy_percent</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>pmi</t>
+          <t>display_pmi</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>e_factor</t>
+          <t>display_e_factor</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>overall_yield_percent_from_summary</t>
+          <t>display_overall_yield_percent</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>overall_yield_percent_from_steps</t>
+          <t>display_number_of_steps</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
         <is>
-          <t>number_of_steps</t>
+          <t>average_hazard_score</t>
         </is>
       </c>
       <c r="K1" t="inlineStr">
         <is>
-          <t>step_penalty</t>
+          <t>recommended_solvents_count</t>
         </is>
       </c>
       <c r="L1" t="inlineStr">
         <is>
-          <t>average_hazard_score</t>
+          <t>problematic_solvents_count</t>
         </is>
       </c>
       <c r="M1" t="inlineStr">
         <is>
-          <t>solvent_summary</t>
+          <t>hazardous_solvents_count</t>
         </is>
       </c>
       <c r="N1" t="inlineStr">
         <is>
-          <t>solvent_details</t>
+          <t>overall_solvent_profile</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>app_value_source</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>calculation_basis</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>data_confidence</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>app_notes</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>calculated_atom_economy_percent</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>calculated_pmi</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>calculated_e_factor</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>calculated_stepwise_yield_percent</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>pmi_calc_status</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>efactor_calc_status</t>
         </is>
       </c>
     </row>
@@ -510,33 +560,73 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>33.22509567435927</v>
-      </c>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
+        <v>77</v>
+      </c>
+      <c r="F2" t="n">
+        <v>3.34</v>
+      </c>
+      <c r="G2" t="n">
+        <v>2.34</v>
+      </c>
       <c r="H2" t="n">
         <v>52.1</v>
       </c>
       <c r="I2" t="n">
-        <v>52.12698400000001</v>
+        <v>3</v>
       </c>
       <c r="J2" t="n">
-        <v>3</v>
+        <v>3.33</v>
       </c>
       <c r="K2" t="n">
-        <v>0.8573749999999999</v>
+        <v>0</v>
       </c>
       <c r="L2" t="n">
-        <v>3.333333333333333</v>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>{}</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>[]</t>
+        <v>0</v>
+      </c>
+      <c r="M2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>Use reference values</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>Reference / simplified route estimate; raw workbook masses are not on one consistent route scale.</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>Use these for the missing PMI/E-factor instead of leaving blanks.</t>
+        </is>
+      </c>
+      <c r="S2" t="n">
+        <v>33.23</v>
+      </c>
+      <c r="T2" t="n">
+        <v>45.28</v>
+      </c>
+      <c r="U2" t="n">
+        <v>44.28</v>
+      </c>
+      <c r="V2" t="n">
+        <v>52.13</v>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>ok</t>
         </is>
       </c>
     </row>
@@ -562,33 +652,77 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>18.2025148908008</v>
-      </c>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
+        <v>28.5</v>
+      </c>
+      <c r="F3" t="n">
+        <v>26.4</v>
+      </c>
+      <c r="G3" t="n">
+        <v>25.4</v>
+      </c>
       <c r="H3" t="n">
+        <v>88.3</v>
+      </c>
+      <c r="I3" t="n">
+        <v>3</v>
+      </c>
+      <c r="J3" t="n">
+        <v>2.82</v>
+      </c>
+      <c r="K3" t="n">
+        <v>3</v>
+      </c>
+      <c r="L3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>Recommended</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>Use reference values</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>Reference / simplified route estimate; process-model route.</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>Use these for missing PMI/E-factor; final API/product basis should be clearly labelled.</t>
+        </is>
+      </c>
+      <c r="S3" t="n">
+        <v>18.2</v>
+      </c>
+      <c r="T3" t="n">
+        <v>808.1799999999999</v>
+      </c>
+      <c r="U3" t="n">
+        <v>807.1799999999999</v>
+      </c>
+      <c r="V3" t="n">
         <v>88.29000000000001</v>
       </c>
-      <c r="I3" t="n">
-        <v>88.2882</v>
-      </c>
-      <c r="J3" t="n">
-        <v>3</v>
-      </c>
-      <c r="K3" t="n">
-        <v>0.8573749999999999</v>
-      </c>
-      <c r="L3" t="n">
-        <v>2.818181818181818</v>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>{'Recommended': 3}</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>[{'solvent': 'Methanol', 'score': 3, 'category': 'Recommended'}, {'solvent': 'Methanol', 'score': 3, 'category': 'Recommended'}, {'solvent': 'Water', 'score': 1, 'category': 'Recommended'}]</t>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="X3" t="inlineStr">
+        <is>
+          <t>ok</t>
         </is>
       </c>
     </row>
@@ -614,37 +748,77 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>10.50822767355194</v>
+        <v>10.51</v>
       </c>
       <c r="F4" t="n">
-        <v>916.520634920635</v>
+        <v>25</v>
       </c>
       <c r="G4" t="n">
-        <v>915.520634920635</v>
+        <v>24</v>
       </c>
       <c r="H4" t="n">
         <v>9</v>
       </c>
       <c r="I4" t="n">
-        <v>8.908073999999999</v>
+        <v>9</v>
       </c>
       <c r="J4" t="n">
-        <v>5</v>
+        <v>2.31</v>
       </c>
       <c r="K4" t="n">
-        <v>0.7737809374999998</v>
+        <v>2</v>
       </c>
       <c r="L4" t="n">
-        <v>2.307692307692307</v>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>{'Problematic': 1, 'Recommended': 2}</t>
-        </is>
+        <v>1</v>
+      </c>
+      <c r="M4" t="n">
+        <v>0</v>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>[{'solvent': 'Toluene', 'score': 6, 'category': 'Problematic'}, {'solvent': 'Methanol', 'score': 3, 'category': 'Recommended'}, {'solvent': 'Water', 'score': 1, 'category': 'Recommended'}]</t>
+          <t>Problematic</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>Curated comparator value</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>Curated route-comparison estimate</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>Display PMI/E-factor set to a curated route-comparison value.</t>
+        </is>
+      </c>
+      <c r="S4" t="n">
+        <v>10.51</v>
+      </c>
+      <c r="T4" t="n">
+        <v>459.1</v>
+      </c>
+      <c r="U4" t="n">
+        <v>458.1</v>
+      </c>
+      <c r="V4" t="n">
+        <v>8.91</v>
+      </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="X4" t="inlineStr">
+        <is>
+          <t>ok</t>
         </is>
       </c>
     </row>
@@ -670,37 +844,77 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>10.69354255317134</v>
+        <v>10.69</v>
       </c>
       <c r="F5" t="n">
-        <v>159622</v>
+        <v>60</v>
       </c>
       <c r="G5" t="n">
-        <v>159621</v>
+        <v>59</v>
       </c>
       <c r="H5" t="n">
         <v>0.5</v>
       </c>
       <c r="I5" t="n">
-        <v>0.51906645504</v>
+        <v>9</v>
       </c>
       <c r="J5" t="n">
-        <v>10</v>
+        <v>2.23</v>
       </c>
       <c r="K5" t="n">
-        <v>0.5987369392383787</v>
+        <v>1</v>
       </c>
       <c r="L5" t="n">
-        <v>2.225806451612903</v>
-      </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>{'Problematic': 2, 'Recommended': 1}</t>
-        </is>
+        <v>2</v>
+      </c>
+      <c r="M5" t="n">
+        <v>0</v>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>[{'solvent': 'THF', 'score': 6, 'category': 'Problematic'}, {'solvent': 'Acetone', 'score': 3, 'category': 'Recommended'}, {'solvent': 'Toluene', 'score': 6, 'category': 'Problematic'}]</t>
+          <t>Problematic</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>Curated comparator value</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>Curated route-comparison estimate</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>Display PMI/E-factor set to a curated high-penalty comparator value.</t>
+        </is>
+      </c>
+      <c r="S5" t="n">
+        <v>10.69</v>
+      </c>
+      <c r="T5" t="n">
+        <v>159617.48</v>
+      </c>
+      <c r="U5" t="n">
+        <v>159616.48</v>
+      </c>
+      <c r="V5" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="W5" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="X5" t="inlineStr">
+        <is>
+          <t>ok</t>
         </is>
       </c>
     </row>
@@ -726,33 +940,77 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>4.984656213377324</v>
-      </c>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
+        <v>4.98</v>
+      </c>
+      <c r="F6" t="n">
+        <v>6</v>
+      </c>
+      <c r="G6" t="n">
+        <v>5</v>
+      </c>
       <c r="H6" t="n">
+        <v>5</v>
+      </c>
+      <c r="I6" t="n">
+        <v>13</v>
+      </c>
+      <c r="J6" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="K6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" t="n">
         <v>3</v>
       </c>
-      <c r="I6" t="n">
-        <v>3.1931865</v>
-      </c>
-      <c r="J6" t="n">
-        <v>10</v>
-      </c>
-      <c r="K6" t="n">
-        <v>0.5987369392383787</v>
-      </c>
-      <c r="L6" t="n">
-        <v>2.6</v>
-      </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>{'Problematic': 3}</t>
-        </is>
+      <c r="M6" t="n">
+        <v>0</v>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>[{'solvent': 'THF', 'score': 6, 'category': 'Problematic'}, {'solvent': 'THF', 'score': 6, 'category': 'Problematic'}, {'solvent': 'THF', 'score': 6, 'category': 'Problematic'}]</t>
+          <t>Problematic</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>Curated comparator value</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>Curated route-comparison estimate</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>Display PMI/E-factor set to a curated comparator value.</t>
+        </is>
+      </c>
+      <c r="S6" t="n">
+        <v>4.98</v>
+      </c>
+      <c r="T6" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="U6" t="n">
+        <v>-0.55</v>
+      </c>
+      <c r="V6" t="n">
+        <v>3.19</v>
+      </c>
+      <c r="W6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="X6" t="inlineStr">
+        <is>
+          <t>ok</t>
         </is>
       </c>
     </row>
@@ -778,33 +1036,77 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>20.25525320860027</v>
-      </c>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr"/>
+        <v>20.26</v>
+      </c>
+      <c r="F7" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="G7" t="n">
+        <v>1.2</v>
+      </c>
       <c r="H7" t="n">
-        <v>40</v>
+        <v>55</v>
       </c>
       <c r="I7" t="n">
-        <v>40.96575</v>
+        <v>5</v>
       </c>
       <c r="J7" t="n">
-        <v>5</v>
+        <v>1.61</v>
       </c>
       <c r="K7" t="n">
-        <v>0.7737809374999998</v>
+        <v>1</v>
       </c>
       <c r="L7" t="n">
-        <v>1.611111111111111</v>
-      </c>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>{'Recommended': 1}</t>
-        </is>
+        <v>0</v>
+      </c>
+      <c r="M7" t="n">
+        <v>0</v>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>[{'solvent': 'Methanol', 'score': 3, 'category': 'Recommended'}]</t>
+          <t>Recommended</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>Curated comparator value</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>Curated semi-synthetic comparator value</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>Display PMI/E-factor set to a curated comparator value.</t>
+        </is>
+      </c>
+      <c r="S7" t="n">
+        <v>20.26</v>
+      </c>
+      <c r="T7" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="U7" t="n">
+        <v>-0.66</v>
+      </c>
+      <c r="V7" t="n">
+        <v>40.97</v>
+      </c>
+      <c r="W7" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="X7" t="inlineStr">
+        <is>
+          <t>ok</t>
         </is>
       </c>
     </row>
@@ -830,37 +1132,73 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>73.97104595839235</v>
+        <v>73.90000000000001</v>
       </c>
       <c r="F8" t="n">
-        <v>1.351880302682871</v>
+        <v>1.48</v>
       </c>
       <c r="G8" t="n">
-        <v>0.3518803026828708</v>
+        <v>0.48</v>
       </c>
       <c r="H8" t="n">
         <v>67.5</v>
       </c>
       <c r="I8" t="n">
-        <v>44.14558176</v>
+        <v>5</v>
       </c>
       <c r="J8" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="K8" t="n">
-        <v>0.7737809374999998</v>
+        <v>0</v>
       </c>
       <c r="L8" t="n">
-        <v>3</v>
-      </c>
-      <c r="M8" t="inlineStr">
-        <is>
-          <t>{}</t>
-        </is>
-      </c>
-      <c r="N8" t="inlineStr">
-        <is>
-          <t>[]</t>
+        <v>0</v>
+      </c>
+      <c r="M8" t="n">
+        <v>0</v>
+      </c>
+      <c r="N8" t="inlineStr"/>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>Use reference/theoretical minimum</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>Reference / theoretical minimum basis.</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>PMI/E-factor are theoretical minima; label clearly in app.</t>
+        </is>
+      </c>
+      <c r="S8" t="n">
+        <v>73.97</v>
+      </c>
+      <c r="T8" t="n">
+        <v>2.12</v>
+      </c>
+      <c r="U8" t="n">
+        <v>1.12</v>
+      </c>
+      <c r="V8" t="n">
+        <v>44.15</v>
+      </c>
+      <c r="W8" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="X8" t="inlineStr">
+        <is>
+          <t>ok</t>
         </is>
       </c>
     </row>
@@ -886,37 +1224,73 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>90.0072236937154</v>
+        <v>90.01000000000001</v>
       </c>
       <c r="F9" t="n">
-        <v>1.111021936864633</v>
+        <v>1.31</v>
       </c>
       <c r="G9" t="n">
-        <v>0.1110219368646333</v>
+        <v>0.31</v>
       </c>
       <c r="H9" t="n">
         <v>76.28</v>
       </c>
       <c r="I9" t="n">
-        <v>76.2804</v>
+        <v>2</v>
       </c>
       <c r="J9" t="n">
-        <v>2</v>
+        <v>1.6</v>
       </c>
       <c r="K9" t="n">
-        <v>0.9025</v>
+        <v>0</v>
       </c>
       <c r="L9" t="n">
-        <v>1.6</v>
-      </c>
-      <c r="M9" t="inlineStr">
-        <is>
-          <t>{}</t>
-        </is>
-      </c>
-      <c r="N9" t="inlineStr">
-        <is>
-          <t>[]</t>
+        <v>0</v>
+      </c>
+      <c r="M9" t="n">
+        <v>0</v>
+      </c>
+      <c r="N9" t="inlineStr"/>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>Use reference/theoretical minimum</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>Reference / theoretical minimum basis.</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>Matches current atom economy/yield closely; use as app display values.</t>
+        </is>
+      </c>
+      <c r="S9" t="n">
+        <v>90.01000000000001</v>
+      </c>
+      <c r="T9" t="n">
+        <v>1.28</v>
+      </c>
+      <c r="U9" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="V9" t="n">
+        <v>76.28</v>
+      </c>
+      <c r="W9" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="X9" t="inlineStr">
+        <is>
+          <t>ok</t>
         </is>
       </c>
     </row>
@@ -942,37 +1316,77 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>95.01852180471141</v>
+        <v>95.02</v>
       </c>
       <c r="F10" t="n">
-        <v>1.052426391199043</v>
+        <v>1.41</v>
       </c>
       <c r="G10" t="n">
-        <v>0.05242639119904289</v>
+        <v>0.41</v>
       </c>
       <c r="H10" t="n">
         <v>74.64</v>
       </c>
       <c r="I10" t="n">
-        <v>74.640336</v>
+        <v>4</v>
       </c>
       <c r="J10" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="K10" t="n">
         <v>4</v>
       </c>
-      <c r="K10" t="n">
-        <v>0.8145062499999999</v>
-      </c>
       <c r="L10" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="M10" t="inlineStr">
-        <is>
-          <t>{'Problematic': 1, 'Recommended': 4}</t>
-        </is>
+        <v>1</v>
+      </c>
+      <c r="M10" t="n">
+        <v>0</v>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>[{'solvent': 'Acetonitrile', 'score': 5, 'category': 'Problematic'}, {'solvent': 'Methanol', 'score': 3, 'category': 'Recommended'}, {'solvent': 'Ethanol', 'score': 2, 'category': 'Recommended'}, {'solvent': 'Ethanol', 'score': 2, 'category': 'Recommended'}, {'solvent': 'Ethanol', 'score': 2, 'category': 'Recommended'}]</t>
+          <t>Problematic</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>Use reference values</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>Reference values provided by user; final product mass basis included.</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>Use reference PMI/E-factor because workbook calculated values were too low.</t>
+        </is>
+      </c>
+      <c r="S10" t="n">
+        <v>95.02</v>
+      </c>
+      <c r="T10" t="n">
+        <v>1.32</v>
+      </c>
+      <c r="U10" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="V10" t="n">
+        <v>74.64</v>
+      </c>
+      <c r="W10" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="X10" t="inlineStr">
+        <is>
+          <t>ok</t>
         </is>
       </c>
     </row>
@@ -998,37 +1412,159 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>61.91968618570042</v>
+        <v>61.91</v>
       </c>
       <c r="F11" t="n">
-        <v>1.614995264996898</v>
+        <v>10.09</v>
       </c>
       <c r="G11" t="n">
-        <v>0.6149952649968977</v>
+        <v>9.09</v>
       </c>
       <c r="H11" t="n">
         <v>16</v>
       </c>
       <c r="I11" t="n">
-        <v>16.00294</v>
+        <v>3</v>
       </c>
       <c r="J11" t="n">
-        <v>3</v>
+        <v>2.33</v>
       </c>
       <c r="K11" t="n">
-        <v>0.8573749999999999</v>
+        <v>1</v>
       </c>
       <c r="L11" t="n">
-        <v>2.333333333333333</v>
-      </c>
-      <c r="M11" t="inlineStr">
-        <is>
-          <t>{'Problematic': 1, 'Recommended': 1}</t>
-        </is>
+        <v>1</v>
+      </c>
+      <c r="M11" t="n">
+        <v>0</v>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>[{'solvent': 'Trifluorotoluene', 'score': 6, 'category': 'Problematic'}, {'solvent': 'Methanol', 'score': 3, 'category': 'Recommended'}]</t>
+          <t>Problematic</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>Use reference values</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>Reference values provided by user; final product mass basis included.</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>Use reference PMI/E-factor; previous calculated values undercount route inputs.</t>
+        </is>
+      </c>
+      <c r="S11" t="n">
+        <v>61.92</v>
+      </c>
+      <c r="T11" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="U11" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="V11" t="n">
+        <v>16</v>
+      </c>
+      <c r="W11" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+      <c r="X11" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Ibuprofen</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>IBU_Boots_6STEP</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Boots process</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Ibuprofen</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>40</v>
+      </c>
+      <c r="F12" t="n">
+        <v>121.53</v>
+      </c>
+      <c r="G12" t="n">
+        <v>120.53</v>
+      </c>
+      <c r="H12" t="n">
+        <v>40</v>
+      </c>
+      <c r="I12" t="n">
+        <v>6</v>
+      </c>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="n">
+        <v>0</v>
+      </c>
+      <c r="L12" t="n">
+        <v>0</v>
+      </c>
+      <c r="M12" t="n">
+        <v>0</v>
+      </c>
+      <c r="N12" t="inlineStr"/>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>Historical literature/reference comparator</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>Reference display value</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>Use as a historical comparator against BHC and flow routes.</t>
+        </is>
+      </c>
+      <c r="S12" t="inlineStr"/>
+      <c r="T12" t="inlineStr"/>
+      <c r="U12" t="inlineStr"/>
+      <c r="V12" t="inlineStr"/>
+      <c r="W12" t="inlineStr">
+        <is>
+          <t>No steps available</t>
+        </is>
+      </c>
+      <c r="X12" t="inlineStr">
+        <is>
+          <t>No steps available</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
i cleaned the pipeline code with docstrings and updated final workbook
</commit_message>
<xml_diff>
--- a/data/results/calculated_green_metrics.xlsx
+++ b/data/results/calculated_green_metrics.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X12"/>
+  <dimension ref="A1:AD12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -464,75 +464,105 @@
       </c>
       <c r="J1" t="inlineStr">
         <is>
+          <t>used_fallback_atom_economy</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>used_fallback_pmi</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>used_fallback_e_factor</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>used_fallback_overall_yield</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>used_fallback_number_of_steps</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
           <t>average_hazard_score</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>recommended_solvents_count</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>problematic_solvents_count</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>hazardous_solvents_count</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>overall_solvent_profile</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>unknown_solvent_count</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
         <is>
           <t>app_value_source</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>calculation_basis</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>data_confidence</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>app_notes</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>calculated_atom_economy_percent</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>calculated_pmi</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>calculated_e_factor</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>calculated_stepwise_yield_percent</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
         <is>
           <t>pmi_calc_status</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="AD1" t="inlineStr">
         <is>
           <t>efactor_calc_status</t>
         </is>
@@ -560,13 +590,13 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>77</v>
+        <v>77.45</v>
       </c>
       <c r="F2" t="n">
-        <v>3.34</v>
+        <v>3.14</v>
       </c>
       <c r="G2" t="n">
-        <v>2.34</v>
+        <v>2.14</v>
       </c>
       <c r="H2" t="n">
         <v>52.1</v>
@@ -574,57 +604,75 @@
       <c r="I2" t="n">
         <v>3</v>
       </c>
-      <c r="J2" t="n">
+      <c r="J2" t="b">
+        <v>0</v>
+      </c>
+      <c r="K2" t="b">
+        <v>0</v>
+      </c>
+      <c r="L2" t="b">
+        <v>0</v>
+      </c>
+      <c r="M2" t="b">
+        <v>0</v>
+      </c>
+      <c r="N2" t="b">
+        <v>0</v>
+      </c>
+      <c r="O2" t="n">
         <v>3.33</v>
       </c>
-      <c r="K2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>Use reference values</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>Reference / simplified route estimate; raw workbook masses are not on one consistent route scale.</t>
-        </is>
-      </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="R2" t="inlineStr">
-        <is>
-          <t>Use these for the missing PMI/E-factor instead of leaving blanks.</t>
-        </is>
-      </c>
-      <c r="S2" t="n">
-        <v>33.23</v>
+      <c r="P2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>1</v>
+      </c>
+      <c r="R2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>Problematic</t>
+        </is>
       </c>
       <c r="T2" t="n">
-        <v>45.28</v>
-      </c>
-      <c r="U2" t="n">
-        <v>44.28</v>
-      </c>
-      <c r="V2" t="n">
+        <v>0</v>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>reference</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>reference estimate</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="X2" t="inlineStr"/>
+      <c r="Y2" t="n">
+        <v>77.45</v>
+      </c>
+      <c r="Z2" t="n">
+        <v>3.14</v>
+      </c>
+      <c r="AA2" t="n">
+        <v>2.14</v>
+      </c>
+      <c r="AB2" t="n">
         <v>52.13</v>
       </c>
-      <c r="W2" t="inlineStr">
+      <c r="AC2" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
       </c>
-      <c r="X2" t="inlineStr">
+      <c r="AD2" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
@@ -666,63 +714,69 @@
       <c r="I3" t="n">
         <v>3</v>
       </c>
-      <c r="J3" t="n">
+      <c r="J3" t="b">
+        <v>1</v>
+      </c>
+      <c r="K3" t="b">
+        <v>1</v>
+      </c>
+      <c r="L3" t="b">
+        <v>1</v>
+      </c>
+      <c r="M3" t="b">
+        <v>1</v>
+      </c>
+      <c r="N3" t="b">
+        <v>1</v>
+      </c>
+      <c r="O3" t="n">
         <v>2.82</v>
       </c>
-      <c r="K3" t="n">
+      <c r="P3" t="n">
         <v>3</v>
       </c>
-      <c r="L3" t="n">
-        <v>0</v>
-      </c>
-      <c r="M3" t="n">
-        <v>0</v>
-      </c>
-      <c r="N3" t="inlineStr">
+      <c r="Q3" t="n">
+        <v>0</v>
+      </c>
+      <c r="R3" t="n">
+        <v>0</v>
+      </c>
+      <c r="S3" t="inlineStr">
         <is>
           <t>Recommended</t>
         </is>
       </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>Use reference values</t>
-        </is>
-      </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>Reference / simplified route estimate; process-model route.</t>
-        </is>
-      </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="R3" t="inlineStr">
-        <is>
-          <t>Use these for missing PMI/E-factor; final API/product basis should be clearly labelled.</t>
-        </is>
-      </c>
-      <c r="S3" t="n">
-        <v>18.2</v>
-      </c>
       <c r="T3" t="n">
-        <v>808.1799999999999</v>
-      </c>
-      <c r="U3" t="n">
-        <v>807.1799999999999</v>
-      </c>
-      <c r="V3" t="n">
-        <v>88.29000000000001</v>
+        <v>0</v>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>reference</t>
+        </is>
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="X3" t="inlineStr">
-        <is>
-          <t>ok</t>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="X3" t="inlineStr"/>
+      <c r="Y3" t="inlineStr"/>
+      <c r="Z3" t="inlineStr"/>
+      <c r="AA3" t="inlineStr"/>
+      <c r="AB3" t="inlineStr"/>
+      <c r="AC3" t="inlineStr">
+        <is>
+          <t>Missing/invalid yield at step 3</t>
+        </is>
+      </c>
+      <c r="AD3" t="inlineStr">
+        <is>
+          <t>Missing/invalid yield at step 3</t>
         </is>
       </c>
     </row>
@@ -748,7 +802,7 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>10.51</v>
+        <v>19.1</v>
       </c>
       <c r="F4" t="n">
         <v>25</v>
@@ -760,65 +814,71 @@
         <v>9</v>
       </c>
       <c r="I4" t="n">
-        <v>9</v>
-      </c>
-      <c r="J4" t="n">
+        <v>5</v>
+      </c>
+      <c r="J4" t="b">
+        <v>1</v>
+      </c>
+      <c r="K4" t="b">
+        <v>1</v>
+      </c>
+      <c r="L4" t="b">
+        <v>1</v>
+      </c>
+      <c r="M4" t="b">
+        <v>1</v>
+      </c>
+      <c r="N4" t="b">
+        <v>1</v>
+      </c>
+      <c r="O4" t="n">
         <v>2.31</v>
       </c>
-      <c r="K4" t="n">
+      <c r="P4" t="n">
         <v>2</v>
       </c>
-      <c r="L4" t="n">
-        <v>1</v>
-      </c>
-      <c r="M4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>Problematic</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>Curated comparator value</t>
-        </is>
-      </c>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t>Curated route-comparison estimate</t>
-        </is>
-      </c>
-      <c r="Q4" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="R4" t="inlineStr">
-        <is>
-          <t>Display PMI/E-factor set to a curated route-comparison value.</t>
-        </is>
-      </c>
-      <c r="S4" t="n">
-        <v>10.51</v>
+      <c r="Q4" t="n">
+        <v>1</v>
+      </c>
+      <c r="R4" t="n">
+        <v>1</v>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>Hazardous</t>
+        </is>
       </c>
       <c r="T4" t="n">
-        <v>459.1</v>
-      </c>
-      <c r="U4" t="n">
-        <v>458.1</v>
-      </c>
-      <c r="V4" t="n">
-        <v>8.91</v>
+        <v>2</v>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>curated</t>
+        </is>
       </c>
       <c r="W4" t="inlineStr">
         <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="X4" t="inlineStr">
-        <is>
-          <t>ok</t>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="X4" t="inlineStr"/>
+      <c r="Y4" t="inlineStr"/>
+      <c r="Z4" t="inlineStr"/>
+      <c r="AA4" t="inlineStr"/>
+      <c r="AB4" t="inlineStr"/>
+      <c r="AC4" t="inlineStr">
+        <is>
+          <t>Missing/invalid yield at step 5</t>
+        </is>
+      </c>
+      <c r="AD4" t="inlineStr">
+        <is>
+          <t>Missing/invalid yield at step 5</t>
         </is>
       </c>
     </row>
@@ -844,7 +904,7 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>10.69</v>
+        <v>25.3</v>
       </c>
       <c r="F5" t="n">
         <v>60</v>
@@ -856,65 +916,71 @@
         <v>0.5</v>
       </c>
       <c r="I5" t="n">
-        <v>9</v>
-      </c>
-      <c r="J5" t="n">
+        <v>10</v>
+      </c>
+      <c r="J5" t="b">
+        <v>1</v>
+      </c>
+      <c r="K5" t="b">
+        <v>1</v>
+      </c>
+      <c r="L5" t="b">
+        <v>1</v>
+      </c>
+      <c r="M5" t="b">
+        <v>1</v>
+      </c>
+      <c r="N5" t="b">
+        <v>1</v>
+      </c>
+      <c r="O5" t="n">
         <v>2.23</v>
       </c>
-      <c r="K5" t="n">
-        <v>1</v>
-      </c>
-      <c r="L5" t="n">
+      <c r="P5" t="n">
         <v>2</v>
       </c>
-      <c r="M5" t="n">
-        <v>0</v>
-      </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>Problematic</t>
-        </is>
-      </c>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>Curated comparator value</t>
-        </is>
-      </c>
-      <c r="P5" t="inlineStr">
-        <is>
-          <t>Curated route-comparison estimate</t>
-        </is>
-      </c>
-      <c r="Q5" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="R5" t="inlineStr">
-        <is>
-          <t>Display PMI/E-factor set to a curated high-penalty comparator value.</t>
-        </is>
-      </c>
-      <c r="S5" t="n">
-        <v>10.69</v>
+      <c r="Q5" t="n">
+        <v>3</v>
+      </c>
+      <c r="R5" t="n">
+        <v>1</v>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>Hazardous</t>
+        </is>
       </c>
       <c r="T5" t="n">
-        <v>159617.48</v>
-      </c>
-      <c r="U5" t="n">
-        <v>159616.48</v>
-      </c>
-      <c r="V5" t="n">
-        <v>0.52</v>
+        <v>0</v>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>curated</t>
+        </is>
       </c>
       <c r="W5" t="inlineStr">
         <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="X5" t="inlineStr">
-        <is>
-          <t>ok</t>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="X5" t="inlineStr"/>
+      <c r="Y5" t="inlineStr"/>
+      <c r="Z5" t="inlineStr"/>
+      <c r="AA5" t="inlineStr"/>
+      <c r="AB5" t="inlineStr"/>
+      <c r="AC5" t="inlineStr">
+        <is>
+          <t>Missing/invalid yield at step 10</t>
+        </is>
+      </c>
+      <c r="AD5" t="inlineStr">
+        <is>
+          <t>Missing/invalid yield at step 10</t>
         </is>
       </c>
     </row>
@@ -940,7 +1006,7 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>4.98</v>
+        <v>7.2</v>
       </c>
       <c r="F6" t="n">
         <v>6</v>
@@ -952,65 +1018,71 @@
         <v>5</v>
       </c>
       <c r="I6" t="n">
-        <v>13</v>
-      </c>
-      <c r="J6" t="n">
+        <v>6</v>
+      </c>
+      <c r="J6" t="b">
+        <v>1</v>
+      </c>
+      <c r="K6" t="b">
+        <v>1</v>
+      </c>
+      <c r="L6" t="b">
+        <v>1</v>
+      </c>
+      <c r="M6" t="b">
+        <v>1</v>
+      </c>
+      <c r="N6" t="b">
+        <v>1</v>
+      </c>
+      <c r="O6" t="n">
         <v>2.6</v>
       </c>
-      <c r="K6" t="n">
-        <v>0</v>
-      </c>
-      <c r="L6" t="n">
+      <c r="P6" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q6" t="n">
         <v>3</v>
       </c>
-      <c r="M6" t="n">
-        <v>0</v>
-      </c>
-      <c r="N6" t="inlineStr">
+      <c r="R6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S6" t="inlineStr">
         <is>
           <t>Problematic</t>
         </is>
       </c>
-      <c r="O6" t="inlineStr">
-        <is>
-          <t>Curated comparator value</t>
-        </is>
-      </c>
-      <c r="P6" t="inlineStr">
-        <is>
-          <t>Curated route-comparison estimate</t>
-        </is>
-      </c>
-      <c r="Q6" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="R6" t="inlineStr">
-        <is>
-          <t>Display PMI/E-factor set to a curated comparator value.</t>
-        </is>
-      </c>
-      <c r="S6" t="n">
-        <v>4.98</v>
-      </c>
       <c r="T6" t="n">
-        <v>0.45</v>
-      </c>
-      <c r="U6" t="n">
-        <v>-0.55</v>
-      </c>
-      <c r="V6" t="n">
-        <v>3.19</v>
+        <v>5</v>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>curated</t>
+        </is>
       </c>
       <c r="W6" t="inlineStr">
         <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="X6" t="inlineStr">
-        <is>
-          <t>ok</t>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="X6" t="inlineStr"/>
+      <c r="Y6" t="inlineStr"/>
+      <c r="Z6" t="inlineStr"/>
+      <c r="AA6" t="inlineStr"/>
+      <c r="AB6" t="inlineStr"/>
+      <c r="AC6" t="inlineStr">
+        <is>
+          <t>Missing/invalid yield at step 6</t>
+        </is>
+      </c>
+      <c r="AD6" t="inlineStr">
+        <is>
+          <t>Missing/invalid yield at step 6</t>
         </is>
       </c>
     </row>
@@ -1036,7 +1108,7 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>20.26</v>
+        <v>89.8</v>
       </c>
       <c r="F7" t="n">
         <v>2.2</v>
@@ -1050,63 +1122,69 @@
       <c r="I7" t="n">
         <v>5</v>
       </c>
-      <c r="J7" t="n">
+      <c r="J7" t="b">
+        <v>1</v>
+      </c>
+      <c r="K7" t="b">
+        <v>1</v>
+      </c>
+      <c r="L7" t="b">
+        <v>1</v>
+      </c>
+      <c r="M7" t="b">
+        <v>1</v>
+      </c>
+      <c r="N7" t="b">
+        <v>1</v>
+      </c>
+      <c r="O7" t="n">
         <v>1.61</v>
       </c>
-      <c r="K7" t="n">
-        <v>1</v>
-      </c>
-      <c r="L7" t="n">
-        <v>0</v>
-      </c>
-      <c r="M7" t="n">
-        <v>0</v>
-      </c>
-      <c r="N7" t="inlineStr">
-        <is>
-          <t>Recommended</t>
-        </is>
-      </c>
-      <c r="O7" t="inlineStr">
-        <is>
-          <t>Curated comparator value</t>
-        </is>
-      </c>
-      <c r="P7" t="inlineStr">
-        <is>
-          <t>Curated semi-synthetic comparator value</t>
-        </is>
-      </c>
-      <c r="Q7" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="R7" t="inlineStr">
-        <is>
-          <t>Display PMI/E-factor set to a curated comparator value.</t>
-        </is>
-      </c>
-      <c r="S7" t="n">
-        <v>20.26</v>
+      <c r="P7" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>0</v>
+      </c>
+      <c r="R7" t="n">
+        <v>1</v>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>Hazardous</t>
+        </is>
       </c>
       <c r="T7" t="n">
-        <v>0.34</v>
-      </c>
-      <c r="U7" t="n">
-        <v>-0.66</v>
-      </c>
-      <c r="V7" t="n">
-        <v>40.97</v>
+        <v>0</v>
+      </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>curated</t>
+        </is>
       </c>
       <c r="W7" t="inlineStr">
         <is>
-          <t>ok</t>
-        </is>
-      </c>
-      <c r="X7" t="inlineStr">
-        <is>
-          <t>ok</t>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="X7" t="inlineStr"/>
+      <c r="Y7" t="inlineStr"/>
+      <c r="Z7" t="inlineStr"/>
+      <c r="AA7" t="inlineStr"/>
+      <c r="AB7" t="inlineStr"/>
+      <c r="AC7" t="inlineStr">
+        <is>
+          <t>Missing/invalid yield at step 5</t>
+        </is>
+      </c>
+      <c r="AD7" t="inlineStr">
+        <is>
+          <t>Missing/invalid yield at step 5</t>
         </is>
       </c>
     </row>
@@ -1132,13 +1210,13 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>73.90000000000001</v>
+        <v>73.97</v>
       </c>
       <c r="F8" t="n">
-        <v>1.48</v>
+        <v>2.12</v>
       </c>
       <c r="G8" t="n">
-        <v>0.48</v>
+        <v>1.12</v>
       </c>
       <c r="H8" t="n">
         <v>67.5</v>
@@ -1146,57 +1224,75 @@
       <c r="I8" t="n">
         <v>5</v>
       </c>
-      <c r="J8" t="n">
+      <c r="J8" t="b">
+        <v>0</v>
+      </c>
+      <c r="K8" t="b">
+        <v>0</v>
+      </c>
+      <c r="L8" t="b">
+        <v>0</v>
+      </c>
+      <c r="M8" t="b">
+        <v>0</v>
+      </c>
+      <c r="N8" t="b">
+        <v>0</v>
+      </c>
+      <c r="O8" t="n">
         <v>3</v>
       </c>
-      <c r="K8" t="n">
-        <v>0</v>
-      </c>
-      <c r="L8" t="n">
-        <v>0</v>
-      </c>
-      <c r="M8" t="n">
-        <v>0</v>
-      </c>
-      <c r="N8" t="inlineStr"/>
-      <c r="O8" t="inlineStr">
-        <is>
-          <t>Use reference/theoretical minimum</t>
-        </is>
-      </c>
-      <c r="P8" t="inlineStr">
-        <is>
-          <t>Reference / theoretical minimum basis.</t>
-        </is>
-      </c>
-      <c r="Q8" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="R8" t="inlineStr">
-        <is>
-          <t>PMI/E-factor are theoretical minima; label clearly in app.</t>
-        </is>
-      </c>
-      <c r="S8" t="n">
+      <c r="P8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>0</v>
+      </c>
+      <c r="R8" t="n">
+        <v>0</v>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>No solvent data</t>
+        </is>
+      </c>
+      <c r="T8" t="n">
+        <v>0</v>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>reference</t>
+        </is>
+      </c>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>theoretical minimum</t>
+        </is>
+      </c>
+      <c r="W8" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="X8" t="inlineStr"/>
+      <c r="Y8" t="n">
         <v>73.97</v>
       </c>
-      <c r="T8" t="n">
+      <c r="Z8" t="n">
         <v>2.12</v>
       </c>
-      <c r="U8" t="n">
+      <c r="AA8" t="n">
         <v>1.12</v>
       </c>
-      <c r="V8" t="n">
+      <c r="AB8" t="n">
         <v>44.15</v>
       </c>
-      <c r="W8" t="inlineStr">
+      <c r="AC8" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
       </c>
-      <c r="X8" t="inlineStr">
+      <c r="AD8" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
@@ -1227,10 +1323,10 @@
         <v>90.01000000000001</v>
       </c>
       <c r="F9" t="n">
-        <v>1.31</v>
+        <v>1.28</v>
       </c>
       <c r="G9" t="n">
-        <v>0.31</v>
+        <v>0.28</v>
       </c>
       <c r="H9" t="n">
         <v>76.28</v>
@@ -1238,57 +1334,75 @@
       <c r="I9" t="n">
         <v>2</v>
       </c>
-      <c r="J9" t="n">
+      <c r="J9" t="b">
+        <v>0</v>
+      </c>
+      <c r="K9" t="b">
+        <v>0</v>
+      </c>
+      <c r="L9" t="b">
+        <v>0</v>
+      </c>
+      <c r="M9" t="b">
+        <v>0</v>
+      </c>
+      <c r="N9" t="b">
+        <v>0</v>
+      </c>
+      <c r="O9" t="n">
         <v>1.6</v>
       </c>
-      <c r="K9" t="n">
-        <v>0</v>
-      </c>
-      <c r="L9" t="n">
-        <v>0</v>
-      </c>
-      <c r="M9" t="n">
-        <v>0</v>
-      </c>
-      <c r="N9" t="inlineStr"/>
-      <c r="O9" t="inlineStr">
-        <is>
-          <t>Use reference/theoretical minimum</t>
-        </is>
-      </c>
-      <c r="P9" t="inlineStr">
-        <is>
-          <t>Reference / theoretical minimum basis.</t>
-        </is>
-      </c>
-      <c r="Q9" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="R9" t="inlineStr">
-        <is>
-          <t>Matches current atom economy/yield closely; use as app display values.</t>
-        </is>
-      </c>
-      <c r="S9" t="n">
+      <c r="P9" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>0</v>
+      </c>
+      <c r="R9" t="n">
+        <v>0</v>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>No solvent data</t>
+        </is>
+      </c>
+      <c r="T9" t="n">
+        <v>0</v>
+      </c>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>reference</t>
+        </is>
+      </c>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>theoretical minimum</t>
+        </is>
+      </c>
+      <c r="W9" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="X9" t="inlineStr"/>
+      <c r="Y9" t="n">
         <v>90.01000000000001</v>
       </c>
-      <c r="T9" t="n">
+      <c r="Z9" t="n">
         <v>1.28</v>
       </c>
-      <c r="U9" t="n">
+      <c r="AA9" t="n">
         <v>0.28</v>
       </c>
-      <c r="V9" t="n">
+      <c r="AB9" t="n">
         <v>76.28</v>
       </c>
-      <c r="W9" t="inlineStr">
+      <c r="AC9" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
       </c>
-      <c r="X9" t="inlineStr">
+      <c r="AD9" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
@@ -1319,10 +1433,10 @@
         <v>95.02</v>
       </c>
       <c r="F10" t="n">
-        <v>1.41</v>
+        <v>1.32</v>
       </c>
       <c r="G10" t="n">
-        <v>0.41</v>
+        <v>0.32</v>
       </c>
       <c r="H10" t="n">
         <v>74.64</v>
@@ -1330,61 +1444,75 @@
       <c r="I10" t="n">
         <v>4</v>
       </c>
-      <c r="J10" t="n">
+      <c r="J10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K10" t="b">
+        <v>0</v>
+      </c>
+      <c r="L10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M10" t="b">
+        <v>0</v>
+      </c>
+      <c r="N10" t="b">
+        <v>0</v>
+      </c>
+      <c r="O10" t="n">
         <v>2.5</v>
       </c>
-      <c r="K10" t="n">
+      <c r="P10" t="n">
         <v>4</v>
       </c>
-      <c r="L10" t="n">
-        <v>1</v>
-      </c>
-      <c r="M10" t="n">
-        <v>0</v>
-      </c>
-      <c r="N10" t="inlineStr">
+      <c r="Q10" t="n">
+        <v>1</v>
+      </c>
+      <c r="R10" t="n">
+        <v>0</v>
+      </c>
+      <c r="S10" t="inlineStr">
         <is>
           <t>Problematic</t>
         </is>
       </c>
-      <c r="O10" t="inlineStr">
-        <is>
-          <t>Use reference values</t>
-        </is>
-      </c>
-      <c r="P10" t="inlineStr">
-        <is>
-          <t>Reference values provided by user; final product mass basis included.</t>
-        </is>
-      </c>
-      <c r="Q10" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="R10" t="inlineStr">
-        <is>
-          <t>Use reference PMI/E-factor because workbook calculated values were too low.</t>
-        </is>
-      </c>
-      <c r="S10" t="n">
+      <c r="T10" t="n">
+        <v>0</v>
+      </c>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>reference</t>
+        </is>
+      </c>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>reference value</t>
+        </is>
+      </c>
+      <c r="W10" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="X10" t="inlineStr"/>
+      <c r="Y10" t="n">
         <v>95.02</v>
       </c>
-      <c r="T10" t="n">
+      <c r="Z10" t="n">
         <v>1.32</v>
       </c>
-      <c r="U10" t="n">
+      <c r="AA10" t="n">
         <v>0.32</v>
       </c>
-      <c r="V10" t="n">
+      <c r="AB10" t="n">
         <v>74.64</v>
       </c>
-      <c r="W10" t="inlineStr">
+      <c r="AC10" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
       </c>
-      <c r="X10" t="inlineStr">
+      <c r="AD10" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
@@ -1412,13 +1540,13 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>61.91</v>
+        <v>61.92</v>
       </c>
       <c r="F11" t="n">
-        <v>10.09</v>
+        <v>1.8</v>
       </c>
       <c r="G11" t="n">
-        <v>9.09</v>
+        <v>0.8</v>
       </c>
       <c r="H11" t="n">
         <v>16</v>
@@ -1426,61 +1554,75 @@
       <c r="I11" t="n">
         <v>3</v>
       </c>
-      <c r="J11" t="n">
+      <c r="J11" t="b">
+        <v>0</v>
+      </c>
+      <c r="K11" t="b">
+        <v>0</v>
+      </c>
+      <c r="L11" t="b">
+        <v>0</v>
+      </c>
+      <c r="M11" t="b">
+        <v>0</v>
+      </c>
+      <c r="N11" t="b">
+        <v>0</v>
+      </c>
+      <c r="O11" t="n">
         <v>2.33</v>
       </c>
-      <c r="K11" t="n">
-        <v>1</v>
-      </c>
-      <c r="L11" t="n">
-        <v>1</v>
-      </c>
-      <c r="M11" t="n">
-        <v>0</v>
-      </c>
-      <c r="N11" t="inlineStr">
+      <c r="P11" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>1</v>
+      </c>
+      <c r="R11" t="n">
+        <v>0</v>
+      </c>
+      <c r="S11" t="inlineStr">
         <is>
           <t>Problematic</t>
         </is>
       </c>
-      <c r="O11" t="inlineStr">
-        <is>
-          <t>Use reference values</t>
-        </is>
-      </c>
-      <c r="P11" t="inlineStr">
-        <is>
-          <t>Reference values provided by user; final product mass basis included.</t>
-        </is>
-      </c>
-      <c r="Q11" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="R11" t="inlineStr">
-        <is>
-          <t>Use reference PMI/E-factor; previous calculated values undercount route inputs.</t>
-        </is>
-      </c>
-      <c r="S11" t="n">
+      <c r="T11" t="n">
+        <v>2</v>
+      </c>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>reference</t>
+        </is>
+      </c>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>reference value</t>
+        </is>
+      </c>
+      <c r="W11" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="X11" t="inlineStr"/>
+      <c r="Y11" t="n">
         <v>61.92</v>
       </c>
-      <c r="T11" t="n">
+      <c r="Z11" t="n">
         <v>1.8</v>
       </c>
-      <c r="U11" t="n">
+      <c r="AA11" t="n">
         <v>0.8</v>
       </c>
-      <c r="V11" t="n">
+      <c r="AB11" t="n">
         <v>16</v>
       </c>
-      <c r="W11" t="inlineStr">
+      <c r="AC11" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
       </c>
-      <c r="X11" t="inlineStr">
+      <c r="AD11" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
@@ -1522,47 +1664,65 @@
       <c r="I12" t="n">
         <v>6</v>
       </c>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="n">
-        <v>0</v>
-      </c>
-      <c r="L12" t="n">
-        <v>0</v>
-      </c>
-      <c r="M12" t="n">
-        <v>0</v>
-      </c>
-      <c r="N12" t="inlineStr"/>
-      <c r="O12" t="inlineStr">
-        <is>
-          <t>Historical literature/reference comparator</t>
-        </is>
-      </c>
-      <c r="P12" t="inlineStr">
-        <is>
-          <t>Reference display value</t>
-        </is>
-      </c>
-      <c r="Q12" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="R12" t="inlineStr">
-        <is>
-          <t>Use as a historical comparator against BHC and flow routes.</t>
-        </is>
-      </c>
-      <c r="S12" t="inlineStr"/>
-      <c r="T12" t="inlineStr"/>
-      <c r="U12" t="inlineStr"/>
-      <c r="V12" t="inlineStr"/>
+      <c r="J12" t="b">
+        <v>1</v>
+      </c>
+      <c r="K12" t="b">
+        <v>1</v>
+      </c>
+      <c r="L12" t="b">
+        <v>1</v>
+      </c>
+      <c r="M12" t="b">
+        <v>1</v>
+      </c>
+      <c r="N12" t="b">
+        <v>1</v>
+      </c>
+      <c r="O12" t="inlineStr"/>
+      <c r="P12" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>0</v>
+      </c>
+      <c r="R12" t="n">
+        <v>0</v>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>No solvent data</t>
+        </is>
+      </c>
+      <c r="T12" t="n">
+        <v>0</v>
+      </c>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t>historical</t>
+        </is>
+      </c>
       <c r="W12" t="inlineStr">
         <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="X12" t="inlineStr"/>
+      <c r="Y12" t="inlineStr"/>
+      <c r="Z12" t="inlineStr"/>
+      <c r="AA12" t="inlineStr"/>
+      <c r="AB12" t="inlineStr"/>
+      <c r="AC12" t="inlineStr">
+        <is>
           <t>No steps available</t>
         </is>
       </c>
-      <c r="X12" t="inlineStr">
+      <c r="AD12" t="inlineStr">
         <is>
           <t>No steps available</t>
         </is>

</xml_diff>